<commit_message>
CORRECAO C-2 - LIMITE DE VALIDACAO DE DATA NA ABA INICIO
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/GESTAO_DE_OBRAS_OBRA_MODELO_V8.xlsx
+++ b/dados/GESTAO_DE_OBRAS_OBRA_MODELO_V8.xlsx
@@ -774,10 +774,10 @@
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Data inválida" error="Informe uma data válida." type="date" operator="greaterThanOrEqual">
-      <formula1>1900-01-01</formula1>
+      <formula1>DATE(1900,1,1)</formula1>
     </dataValidation>
     <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Data inválida" error="Informe uma data válida." type="date" operator="greaterThanOrEqual">
-      <formula1>1900-01-01</formula1>
+      <formula1>DATE(1900,1,1)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>